<commit_message>
Regenerate complete execution and comparison workbooks
Co-authored-by: DMSILVA87 <DMSILVA87@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PDN_2023-2027_Angola/01_Execucao_PDN_2025.xlsx
+++ b/PDN_2023-2027_Angola/01_Execucao_PDN_2025.xlsx
@@ -17,12 +17,12 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leia-me'!$A$1:$B$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Indicadores_Execução'!$A$1:$P$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Indicadores_Execução'!$A$1:$S$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Índice_Domínios'!$A$1:$E$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ações_2025'!$A$1:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Estrutura_Programa'!$A$1:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Resumo_Execução'!$A$1:$E$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Manifesto_Fontes'!$A$1:$E$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Manifesto_Fontes'!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -184,9 +184,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_indicadores_execucao" displayName="T_indicadores_execucao" ref="A1:P8" headerRowCount="1">
-  <autoFilter ref="A1:P8"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_indicadores_execucao" displayName="T_indicadores_execucao" ref="A1:S52" headerRowCount="1">
+  <autoFilter ref="A1:S52"/>
+  <tableColumns count="19">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Domínio"/>
     <tableColumn id="3" name="Indicador"/>
@@ -194,15 +194,18 @@
     <tableColumn id="5" name="2022_Base"/>
     <tableColumn id="6" name="2023"/>
     <tableColumn id="7" name="2024"/>
-    <tableColumn id="8" name="2025"/>
-    <tableColumn id="9" name="2022_Base_Original"/>
-    <tableColumn id="10" name="2023_Original"/>
-    <tableColumn id="11" name="2024_Original"/>
-    <tableColumn id="12" name="2025_Original"/>
-    <tableColumn id="13" name="Fonte"/>
-    <tableColumn id="14" name="Fonte URL"/>
-    <tableColumn id="15" name="Estado"/>
-    <tableColumn id="16" name="Observação"/>
+    <tableColumn id="8" name="Meta_2025"/>
+    <tableColumn id="9" name="2025"/>
+    <tableColumn id="10" name="2022_Base_Original"/>
+    <tableColumn id="11" name="2023_Original"/>
+    <tableColumn id="12" name="2024_Original"/>
+    <tableColumn id="13" name="Meta_2025_Original"/>
+    <tableColumn id="14" name="2025_Original"/>
+    <tableColumn id="15" name="Fonte"/>
+    <tableColumn id="16" name="Fonte URL"/>
+    <tableColumn id="17" name="Fonte Bundle URL"/>
+    <tableColumn id="18" name="Estado"/>
+    <tableColumn id="19" name="Observação"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -267,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T_manifesto_fontes" displayName="T_manifesto_fontes" ref="A1:E3" headerRowCount="1">
-  <autoFilter ref="A1:E3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T_manifesto_fontes" displayName="T_manifesto_fontes" ref="A1:E4" headerRowCount="1">
+  <autoFilter ref="A1:E4"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Fonte"/>
     <tableColumn id="2" name="URL solicitada"/>
@@ -680,31 +683,31 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Todos os sete separadores de domínio foram verificados no HTML.</t>
+          <t>Todos os sete separadores de domínio foram verificados no HTML e no bundle JavaScript lazy associado.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Limitação principal</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Só Saúde contém tabela de indicadores no HTML publicado; os outros seis separadores estão vazios.</t>
+          <t>Fonte técnica dos indicadores</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Tratamento de ausência</t>
+          <t>Tratamento de carregamento</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Sem dados publicados não foi convertido em zero.</t>
+          <t>Os separadores inactivos são lazy-loaded; os 51 indicadores foram extraídos do bundle oficial.</t>
         </is>
       </c>
     </row>
@@ -737,6 +740,7 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -757,25 +761,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:S52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="45" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="48" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="18" max="18"/>
+    <col width="58" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -816,45 +823,60 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Meta_2025</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2022_Base_Original</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2023_Original</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>2024_Original</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Meta_2025_Original</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>2025_Original</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Fonte</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Fonte URL</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Fonte Bundle URL</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
@@ -890,47 +912,58 @@
       <c r="G2" s="5" t="n">
         <v>7019</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="5" t="n">
         <v>7304</v>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>5 250</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>5 763</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>7 019</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>7 304</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>MINSA</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>Extraído</t>
-        </is>
-      </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>* 2022 é o ano base indicado na fonte.</t>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
         </is>
       </c>
     </row>
@@ -965,46 +998,59 @@
         <v>75</v>
       </c>
       <c r="H3" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="I3" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>MINSA</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>Extraído</t>
-        </is>
-      </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>* 2022 é o ano base indicado na fonte.</t>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
         </is>
       </c>
     </row>
@@ -1039,46 +1085,59 @@
         <v>85</v>
       </c>
       <c r="H4" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="I4" s="5" t="n">
         <v>78</v>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>79</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>96</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>85</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>78</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>MINSA</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>Extraído</t>
-        </is>
-      </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>* 2022 é o ano base indicado na fonte.</t>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
         </is>
       </c>
     </row>
@@ -1113,46 +1172,59 @@
         <v>68</v>
       </c>
       <c r="H5" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="I5" s="5" t="n">
         <v>76</v>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>66</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>71</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>68</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>76</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>MINSA</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>Extraído</t>
-        </is>
-      </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>* 2022 é o ano base indicado na fonte.</t>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
         </is>
       </c>
     </row>
@@ -1187,46 +1259,59 @@
         <v>307</v>
       </c>
       <c r="H6" s="5" t="n">
+        <v>215</v>
+      </c>
+      <c r="I6" s="5" t="n">
         <v>298</v>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>255</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>266</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>307</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>298</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>MINSA</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>Extraído</t>
-        </is>
-      </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>* 2022 é o ano base indicado na fonte.</t>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
         </is>
       </c>
     </row>
@@ -1261,46 +1346,59 @@
         <v>74</v>
       </c>
       <c r="H7" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="I7" s="5" t="n">
         <v>91</v>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>67</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>74</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>MINSA</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>Extraído</t>
-        </is>
-      </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>* 2022 é o ano base indicado na fonte.</t>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
         </is>
       </c>
     </row>
@@ -1335,51 +1433,3872 @@
         <v>51</v>
       </c>
       <c r="H8" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="I8" s="5" t="n">
         <v>64</v>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>49</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t>51</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>64</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>MINSA</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
-        </is>
-      </c>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t>Extraído</t>
-        </is>
-      </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>* 2022 é o ano base indicado na fonte.</t>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>IMP-proteccao_social-pessoas_integradas_em_actividades_geradoras_de_renda_cumulativo</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Protecção Social</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Pessoas integradas em actividades geradoras de renda (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>37000</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>37545</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>38289</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>99000</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>38917</v>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>37 000</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>37 545</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>38 289</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>99 000</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>38 917</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>MASFAMU</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>IMP-proteccao_social-beneficiarios_de_transferencias_sociais_monetarias_cumulativo</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Protecção Social</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Beneficiários de transferências sociais monetárias (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>610832</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>951203</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>1070037</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>1350850</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>610 832</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>951 203</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>1 070 037</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>1 800 000</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>1 350 850</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>MASFAMU</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>IMP-proteccao_social-familias_assistidas_com_cesta_basica_de_alimentos_cumulativo</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Protecção Social</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Famílias assistidas com cesta básica de alimentos (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>23070</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>30054</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>90419</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>83000</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>104807</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>23 070</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>30 054</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>90 419</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>83 000</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>104 807</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>MASFAMU</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>IMP-comunicacao-numero_de_assinantes_de_internet</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Comunicação</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Número de assinantes de Internet</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>N.º/100 habitantes</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>MINTTICS</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>IMP-comunicacao-numero_de_assinantes_de_servicos_moveis</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Comunicação</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Número de assinantes de serviços móveis</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>N.º/100 habitantes</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>79</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>MINTTICS</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-salas_de_aula_do_ensino_primario_cumulativo</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Salas de aula do Ensino Primário (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>60004</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>62395</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>61516</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>60018</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>65388</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>60 004</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>62 395</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>61 516</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>60 018</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>65 388</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-salas_de_aula_do_i_ciclo_do_ensino_secundario_cumulativo</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Salas de aula do I Ciclo do Ensino Secundário (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>29323</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>36255</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>42192</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>16286</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>48972</v>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>29 323</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>36 255</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>42 192</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>16 286</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>48 972</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-salas_de_aula_do_ii_ciclo_do_ensino_secundario_cumulativo</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Salas de aula do II Ciclo do Ensino Secundário (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>16409</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>15962</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>19174</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>11141</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>24435</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>16 409</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>15 962</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>19 174</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>11 141</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>24 435</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-taxa_de_alfabetizacao_da_populacao_maior_que_15_anos</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de alfabetização da população maior que 15 anos</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>77</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>INE/MED</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-taxa_de_conclusao_do_ensino_primario</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de conclusão do Ensino Primário</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-taxa_de_conclusao_do_i_ciclo_do_ensino_secundario_ensino_geral</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de conclusão do I Ciclo do Ensino Secundário (Ensino Geral)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-taxa_de_conclusao_do_ii_ciclo_do_ensino_secundario_ensino_geral</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de conclusão do II Ciclo do Ensino Secundário (Ensino Geral)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-professores_de_ensino_pre_escolar_com_a_qualificacao_minima_exigida_cumulativo</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Professores de Ensino Pré-escolar com a qualificação mínima exigida (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-professores_de_ensino_primario_com_a_qualificacao_minima_exigida_cumulativo</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Professores de Ensino Primário com a qualificação mínima exigida (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>81</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-professores_de_ensino_secundario_com_a_qualificacao_minima_exigida_cumulativo</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Professores de Ensino Secundário com a qualificação mínima exigida (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-numero_de_pessoas_formadas_pelo_snefp_cumulativo</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Número de pessoas formadas pelo SNEFP (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>100194</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>188865</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>341490</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>353000</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>524016</v>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>100 194</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>188 865</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>341 490</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>353 000</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>524 016</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>UTGPNFQ</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-kits_profissionais_distribuidos_cumulativo</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Kits profissionais distribuídos (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>25483</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>27131</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>27580</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>27580</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>28070</v>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>25 483</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>27 131</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>27 580</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>27 580</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>28 070</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>MAPTSS</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R25" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>IMP-educacao_e_formacao_profissional-estudantes_matriculados_no_ensino_superior_cumulativo</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Educação e Formação Profissional</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Estudantes matriculados no Ensino Superior (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>320432</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>334842</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>343235</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>411774</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>329548</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>320 432</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>334 842</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>343 235</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>411 774</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>329 548</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>MESCTI</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-estradas_nacionais_reabilitadas_cumulativo</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Estradas Nacionais reabilitadas (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Km</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>9474</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>9924</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>10121</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>10424</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>10338.64</v>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>9 474</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>9 924</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>10 121</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>10 424</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>10 338,64</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>MINOPUH</t>
+        </is>
+      </c>
+      <c r="P27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R27" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S27" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-equipamentos_sociais_construidos_ou_reabilitados_cumulativo</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Equipamentos sociais construídos ou reabilitados (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>151</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>167</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>801</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>204</v>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>801</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>MINOPUH</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-construcao_e_reabilitacao_de_pontes_cumulativo</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Construção e reabilitação de pontes (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>3910</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>5360</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>10114</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>5950.5</v>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>3 910</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>4 400</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>5 360</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>10 114</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>5 950,5</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>MINOPUH</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S29" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-taxa_de_electrificacao</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de electrificação</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>% da população</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>MINEA</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-numero_de_ligacoes_cumulativo</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Número de ligações (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Milhões</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>MINEA</t>
+        </is>
+      </c>
+      <c r="P31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R31" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S31" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-numero_de_sedes_municipais_com_distribuicao_de_energia_pela_ende</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Número de sedes municipais com distribuição de energia pela ENDE</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>MINEA</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-de_producao_total_de_energia_de_fontes_renovaveis</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>% de produção total de energia de fontes renováveis</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>MINEA</t>
+        </is>
+      </c>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S33" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-potencia_instalada_proveniente_de_fontes_renovaveis</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Potência instalada proveniente de fontes renováveis</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>MINEA</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-quantidade_de_agua_tratada_cumulativo</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Quantidade de água tratada (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Mm³/d</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>1320</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>1324</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>1630</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>1 320</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>1 324</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>1 325</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>1 630</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>1 325</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>MINEA</t>
+        </is>
+      </c>
+      <c r="P35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R35" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S35" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-taxa_de_cobertura_de_aguas_nas_areas_urbanas</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de cobertura de águas nas áreas urbanas</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="H36" s="3" t="n"/>
+      <c r="I36" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>MINEA</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R36" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S36" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>IMP-infraestruturas_habitacao_e_servicos_comunitarios-taxa_de_cobertura_de_aguas_nas_areas_rurais</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Habitação e Serviços Comunitários</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de cobertura de águas nas áreas rurais</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
+          <t>MINEA</t>
+        </is>
+      </c>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R37" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-toneladas_de_carne_produzidas</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas de carne produzidas</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>319962</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>341943</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>333238</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>531444</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>357668</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>319 962</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>341 943</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>333 238</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>531 444</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="inlineStr">
+        <is>
+          <t>357 668</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>MINAGRIF</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R38" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-toneladas_de_raizes_e_tuberculos_produzidas</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas de raízes e tubérculos produzidas</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>12922711</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>13743973</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>14582355</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>17311162</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>16131827</v>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>12 922 711</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>13 743 973</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>14 582 355</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>17 311 162</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="inlineStr">
+        <is>
+          <t>16 131 827</t>
+        </is>
+      </c>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>MINAGRIF</t>
+        </is>
+      </c>
+      <c r="P39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R39" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S39" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-toneladas_de_fruta_produzidas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas de fruta produzidas</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>6079785</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>6487767</v>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>6896497</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>7851527</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>7278221</v>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>6 079 785</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>6 487 767</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>6 896 497</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>7 851 527</t>
+        </is>
+      </c>
+      <c r="N40" s="3" t="inlineStr">
+        <is>
+          <t>7 278 221</t>
+        </is>
+      </c>
+      <c r="O40" s="3" t="inlineStr">
+        <is>
+          <t>MINAGRIF</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R40" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S40" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-toneladas_de_cereais_produzidas</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas de cereais produzidas</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>3187951</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>3357136</v>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>3521636</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>7903325</v>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>3763948</v>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>3 187 951</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>3 357 136</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>3 521 636</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>7 903 325</t>
+        </is>
+      </c>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>3 763 948</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>MINAGRIF</t>
+        </is>
+      </c>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R41" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S41" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-toneladas_de_horticolas_produzidas</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas de hortícolas produzidas</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>1975867</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>2203362</v>
+      </c>
+      <c r="G42" s="5" t="n">
+        <v>2359801</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>2373450</v>
+      </c>
+      <c r="I42" s="5" t="n">
+        <v>2552238</v>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>1 975 867</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>2 203 362</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>2 359 801</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>2 373 450</t>
+        </is>
+      </c>
+      <c r="N42" s="3" t="inlineStr">
+        <is>
+          <t>2 552 238</t>
+        </is>
+      </c>
+      <c r="O42" s="3" t="inlineStr">
+        <is>
+          <t>MINAGRIF</t>
+        </is>
+      </c>
+      <c r="P42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R42" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S42" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-ovos_produzidos</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Ovos produzidos</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Milhões</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>2694</v>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>2761</v>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>2422</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>2981</v>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>2545</v>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>2 694</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>2 761</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>2 422</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>2 981</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t>2 545</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>MINAGRIF</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R43" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S43" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-litros_de_leite_produzidos</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Litros de leite produzidos</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Milhões de Litros</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N44" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O44" s="3" t="inlineStr">
+        <is>
+          <t>MINAGRIF</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R44" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S44" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-unidades_industriais_no_subsector_da_industria_pesqueira_e_de_transformacao_de_carne_instaladas_cumulativo</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Unidades industriais no subsector da indústria pesqueira e de transformação de carne instaladas (cumulativo)</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="O45" s="3" t="inlineStr">
+        <is>
+          <t>MINDCOM</t>
+        </is>
+      </c>
+      <c r="P45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R45" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S45" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>IMP-fomento_a_producao-toneladas_de_peixe_de_captura_industrial_e_semi_industrial_produzidas</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Fomento à Produção</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Toneladas de peixe de captura industrial e semi-industrial produzidas</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Milhares de Toneladas</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>335</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>346</v>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>374</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>357</v>
+      </c>
+      <c r="I46" s="5" t="n">
+        <v>273</v>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>335</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>346</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>374</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>357</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="inlineStr">
+        <is>
+          <t>273</t>
+        </is>
+      </c>
+      <c r="O46" s="3" t="inlineStr">
+        <is>
+          <t>MINPERMAR</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R46" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>IMP-economico-taxa_de_crescimento_do_pib</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de crescimento do PIB</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I47" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N47" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="O47" s="3" t="inlineStr">
+        <is>
+          <t>INE/MINPLAN</t>
+        </is>
+      </c>
+      <c r="P47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R47" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S47" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>IMP-economico-taxa_de_crescimento_do_pib_nao_petrolifero</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de crescimento do PIB não petrolífero</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N48" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="O48" s="3" t="inlineStr">
+        <is>
+          <t>INE/MINPLAN</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R48" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S48" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>IMP-economico-taxa_de_inflacao</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de inflação</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="G49" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="H49" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="I49" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="N49" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="O49" s="3" t="inlineStr">
+        <is>
+          <t>INE</t>
+        </is>
+      </c>
+      <c r="P49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R49" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S49" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>IMP-economico-empregos_formais_bruto_gerados</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Empregos Formais Bruto Gerados</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>193078</v>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>191800</v>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>225157</v>
+      </c>
+      <c r="H50" s="3" t="n"/>
+      <c r="I50" s="5" t="n">
+        <v>220509</v>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>193 078</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>191 800</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
+        <is>
+          <t>225 157</t>
+        </is>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N50" s="3" t="inlineStr">
+        <is>
+          <t>220 509</t>
+        </is>
+      </c>
+      <c r="O50" s="3" t="inlineStr">
+        <is>
+          <t>INSS/MAPTSS</t>
+        </is>
+      </c>
+      <c r="P50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R50" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S50" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>IMP-economico-empregos_formais_liquidos_gerados</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Empregos Formais Líquidos Gerados</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>176966</v>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>182541</v>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>218669</v>
+      </c>
+      <c r="H51" s="3" t="n"/>
+      <c r="I51" s="5" t="n">
+        <v>214264</v>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>176 966</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>182 541</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>218 669</t>
+        </is>
+      </c>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N51" s="3" t="inlineStr">
+        <is>
+          <t>214 264</t>
+        </is>
+      </c>
+      <c r="O51" s="3" t="inlineStr">
+        <is>
+          <t>INSS/MAPTSS</t>
+        </is>
+      </c>
+      <c r="P51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R51" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S51" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>IMP-economico-taxa_de_desemprego</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Taxa de Desemprego</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="I52" s="5" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="N52" s="3" t="inlineStr">
+        <is>
+          <t>26,9</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="inlineStr">
+        <is>
+          <t>INE</t>
+        </is>
+      </c>
+      <c r="P52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/en/publicacoes/relatorios-balanco-pdn</t>
+        </is>
+      </c>
+      <c r="Q52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="inlineStr">
+        <is>
+          <t>Extraído do bundle JavaScript lazy</t>
+        </is>
+      </c>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>* 2022 é o ano base; Meta 2025 é a meta anual publicada no bundle.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P8"/>
+  <autoFilter ref="A1:S52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -1447,7 +5366,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Dados extraídos</t>
+          <t>Dados extraídos do bundle JavaScript lazy</t>
         </is>
       </c>
       <c r="C2" s="5" t="n">
@@ -1455,7 +5374,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Tabela de indicadores presente no HTML renderizado.</t>
+          <t>O painel é lazy-loaded; os valores foram extraídos do bundle oficial associado à página.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -1472,15 +5391,15 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Sem dados publicados no HTML</t>
+          <t>Dados extraídos do bundle JavaScript lazy</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>O separador existe no site, mas o painel recebido não contém tabela nem valores.</t>
+          <t>O painel é lazy-loaded; os valores foram extraídos do bundle oficial associado à página.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1497,15 +5416,15 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Sem dados publicados no HTML</t>
+          <t>Dados extraídos do bundle JavaScript lazy</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>O separador existe no site, mas o painel recebido não contém tabela nem valores.</t>
+          <t>O painel é lazy-loaded; os valores foram extraídos do bundle oficial associado à página.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1522,15 +5441,15 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Sem dados publicados no HTML</t>
+          <t>Dados extraídos do bundle JavaScript lazy</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>O separador existe no site, mas o painel recebido não contém tabela nem valores.</t>
+          <t>O painel é lazy-loaded; os valores foram extraídos do bundle oficial associado à página.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1547,15 +5466,15 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Sem dados publicados no HTML</t>
+          <t>Dados extraídos do bundle JavaScript lazy</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>O separador existe no site, mas o painel recebido não contém tabela nem valores.</t>
+          <t>O painel é lazy-loaded; os valores foram extraídos do bundle oficial associado à página.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1572,15 +5491,15 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Sem dados publicados no HTML</t>
+          <t>Dados extraídos do bundle JavaScript lazy</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>O separador existe no site, mas o painel recebido não contém tabela nem valores.</t>
+          <t>O painel é lazy-loaded; os valores foram extraídos do bundle oficial associado à página.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1597,15 +5516,15 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Sem dados publicados no HTML</t>
+          <t>Dados extraídos do bundle JavaScript lazy</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>O separador existe no site, mas o painel recebido não contém tabela nem valores.</t>
+          <t>O painel é lazy-loaded; os valores foram extraídos do bundle oficial associado à página.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2714,7 +6633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2781,32 +6700,59 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>MINPLAN — bundle JavaScript lazy dos indicadores</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.minplan.gov.ao/_next/static/chunks/c191322d36728caa.js</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>fontes/minplan_indicadores_bundle.js</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>já existente localmente</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>PDN Angola 2023-2027 — AUDA-NEPAD / espelho</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>https://www.nepad.org/sites/default/files/2024-07/20231030%283%29_layout_Final_Angola_PDN%202023-2027-1.pdf</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.nepad.org/sites/default/files/2024-07/20231030%283%29_layout_Final_Angola_PDN%202023-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mpla.ao/wp-content/uploads/2023/12/PDN_Angola_2023-2027.pdf</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>fontes/PDN_Angola_2023-2027.pdf</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>já existente localmente</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>já existente localmente (espelho acessível)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E3"/>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>